<commit_message>
New changes in testrail id
</commit_message>
<xml_diff>
--- a/testcases/taxes/international-tax-setup.xlsx
+++ b/testcases/taxes/international-tax-setup.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="international_tax_setup" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'international_tax_setup'!$A$1:$M$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'international_tax_setup'!$A$1:$M$75</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M87"/>
+  <dimension ref="A1:M75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4111,7 +4111,7 @@
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>One row staged with Apply; KNOWN DEFECT — test.fail(BUG-TAX-IST-002)</t>
+          <t>One row staged with Apply</t>
         </is>
       </c>
       <c r="K52" s="2" t="inlineStr">
@@ -4122,12 +4122,12 @@
       </c>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>Exact text: 'Searching will cause you to lose unsaved changes. Continue?'</t>
+          <t>Unsaved changes dialog: 'Are you sure you want to leave this view? Any unsaved changes will be lost.'</t>
         </is>
       </c>
       <c r="M52" s="2" t="inlineStr">
         <is>
-          <t>NM-4025 trace: TC-IT-34; live copy differs (BUG-TAX-IST-002)</t>
+          <t>NM-4025 trace: TC-IT-34 (shared dialog accepted in place of NM-2395 wording)</t>
         </is>
       </c>
     </row>
@@ -4783,7 +4783,7 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Chronology is checked against a hidden future version, not the displayed row</t>
+          <t>Without a session the page sends the user to sign in</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -4798,15 +4798,13 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>User: automation user (Tax FULL_ACCESS)
-Office: Office 1101 (Corporate)
-Search: Mexico / VAT / Baja California
+          <t>User: none (empty browser context)
 Application: Navigator</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Boundary</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -4826,24 +4824,22 @@
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>Save request held at the network (aborted) — nothing written; needs a future-dated version in the data</t>
+          <t>Page opened fresh; no network mocks; non-mutating</t>
         </is>
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>1. Find row with stored version later than today's
-2. Stage date between them
-3. Save</t>
+          <t>1. Open route with no session</t>
         </is>
       </c>
       <c r="L62" s="2" t="inlineStr">
         <is>
-          <t>Rejected against stored history (skips if no hidden version)</t>
+          <t>Redirect to /auth/sign-in with callbackUrl; no grid</t>
         </is>
       </c>
       <c r="M62" s="2" t="inlineStr">
         <is>
-          <t>NM-4025 trace: TC-IT-28</t>
+          <t>NM-4025 trace: TC-IT-09</t>
         </is>
       </c>
     </row>
@@ -4855,7 +4851,7 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>A past effective date later than the latest stored version saves with HTTP 200</t>
+          <t>Every search and update control has an accessible name</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -4871,19 +4867,19 @@
       <c r="E63" s="2" t="inlineStr">
         <is>
           <t>User: automation user (Tax FULL_ACCESS)
-Office: Office 1101
-Search: IST_WRITE_FIXTURE (disposable)
+Office: Office 1101 (Corporate)
+Search: Mexico / VAT / Baja California
 Application: Navigator</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Persistence</t>
+          <t>Accessibility</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
@@ -4898,24 +4894,22 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>REAL WRITE (insert-only). Runs only with IST_ALLOW_WRITES=true and IST_WRITE_FIXTURE set; fixture must be resettable outside the UI</t>
+          <t>Page opened fresh; no network mocks; non-mutating</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
-          <t>1. Search +5 years
-2. Stage fixture rows at latest+1
-3. Save</t>
+          <t>1. Read accessible names of every control</t>
         </is>
       </c>
       <c r="L63" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200; supplied records only; no error</t>
+          <t>Dates, Rate, commission checkbox and all buttons are named (search dropdowns accepted as-is)</t>
         </is>
       </c>
       <c r="M63" s="2" t="inlineStr">
         <is>
-          <t>NM-4025 trace: TC-IT-25, TC-IT-30</t>
+          <t>WCAG 4.1.2</t>
         </is>
       </c>
     </row>
@@ -4927,7 +4921,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Pending indicators clear and Save is disabled after the successful Save</t>
+          <t>Row checkboxes can be operated with the keyboard</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -4943,19 +4937,19 @@
       <c r="E64" s="2" t="inlineStr">
         <is>
           <t>User: automation user (Tax FULL_ACCESS)
-Office: Office 1101
-Search: IST_WRITE_FIXTURE (disposable)
+Office: Office 1101 (Corporate)
+Search: Mexico / VAT / Baja California
 Application: Navigator</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Persistence</t>
+          <t>Accessibility</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
@@ -4970,22 +4964,23 @@
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>REAL WRITE (insert-only). Runs only with IST_ALLOW_WRITES=true and IST_WRITE_FIXTURE set; fixture must be resettable outside the UI</t>
+          <t>Page opened fresh; no network mocks; non-mutating</t>
         </is>
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>1. Read grid after the Save in 062</t>
+          <t>1. Focus a row checkbox
+2. Press Space twice</t>
         </is>
       </c>
       <c r="L64" s="2" t="inlineStr">
         <is>
-          <t>Nothing pending; Save disabled</t>
+          <t>Selected then cleared</t>
         </is>
       </c>
       <c r="M64" s="2" t="inlineStr">
         <is>
-          <t>NM-4025 trace: TC-IT-31, NM-4005</t>
+          <t>WCAG 2.1.1</t>
         </is>
       </c>
     </row>
@@ -4997,7 +4992,7 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Saved values are returned when searching at or after the new date</t>
+          <t>Tab order through the search panel follows the visual order</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -5013,19 +5008,19 @@
       <c r="E65" s="2" t="inlineStr">
         <is>
           <t>User: automation user (Tax FULL_ACCESS)
-Office: Office 1101
-Search: IST_WRITE_FIXTURE (disposable)
+Office: Office 1101 (Corporate)
+Search: Mexico / VAT / Baja California
 Application: Navigator</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>Persistence</t>
+          <t>Accessibility</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
@@ -5040,23 +5035,23 @@
       </c>
       <c r="J65" s="2" t="inlineStr">
         <is>
-          <t>REAL WRITE (insert-only). Runs only with IST_ALLOW_WRITES=true and IST_WRITE_FIXTURE set; fixture must be resettable outside the UI</t>
+          <t>Page opened fresh; no network mocks; non-mutating</t>
         </is>
       </c>
       <c r="K65" s="2" t="inlineStr">
         <is>
-          <t>1. Search at new date
-2. Search at +5 years</t>
+          <t>1. Focus Country
+2. Tab through the panel</t>
         </is>
       </c>
       <c r="L65" s="2" t="inlineStr">
         <is>
-          <t>Saved rate, flag and date returned</t>
+          <t>Tax Group → Province → Effective Date → Reset → Search</t>
         </is>
       </c>
       <c r="M65" s="2" t="inlineStr">
         <is>
-          <t>NM-4025 trace: TC-IT-32</t>
+          <t>WCAG 2.4.3</t>
         </is>
       </c>
     </row>
@@ -5068,7 +5063,7 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Searching before the new date still returns the previous version</t>
+          <t>No untranslated i18n key is visible on the page</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -5084,19 +5079,19 @@
       <c r="E66" s="2" t="inlineStr">
         <is>
           <t>User: automation user (Tax FULL_ACCESS)
-Office: Office 1101
-Search: IST_WRITE_FIXTURE (disposable)
+Office: Office 1101 (Corporate)
+Search: Mexico / VAT / Baja California
 Application: Navigator</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Persistence</t>
+          <t>Localisation</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
@@ -5111,24 +5106,21 @@
       </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>REAL WRITE (insert-only). Runs only with IST_ALLOW_WRITES=true and IST_WRITE_FIXTURE set; fixture must be resettable outside the UI</t>
+          <t>Page opened fresh; no network mocks; non-mutating</t>
         </is>
       </c>
       <c r="K66" s="2" t="inlineStr">
         <is>
-          <t>1. Search at new date - 1</t>
+          <t>1. Search fixture
+2. Scan page text</t>
         </is>
       </c>
       <c r="L66" s="2" t="inlineStr">
         <is>
-          <t>Pre-save version returned</t>
-        </is>
-      </c>
-      <c r="M66" s="2" t="inlineStr">
-        <is>
-          <t>NM-4025 trace: TC-IT-29</t>
-        </is>
-      </c>
+          <t>No dotted i18n keys</t>
+        </is>
+      </c>
+      <c r="M66" s="2" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -5138,7 +5130,7 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Untouched configurations gain no new versions</t>
+          <t>Automated WCAG 2.1 AA scan finds no serious or critical violations</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
@@ -5154,19 +5146,19 @@
       <c r="E67" s="2" t="inlineStr">
         <is>
           <t>User: automation user (Tax FULL_ACCESS)
-Office: Office 1101
-Search: IST_WRITE_FIXTURE (disposable)
+Office: Office 1101 (Corporate)
+Search: Mexico / VAT / Baja California
 Application: Navigator</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Data integrity</t>
+          <t>Accessibility</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
@@ -5181,23 +5173,23 @@
       </c>
       <c r="J67" s="2" t="inlineStr">
         <is>
-          <t>REAL WRITE (insert-only). Runs only with IST_ALLOW_WRITES=true and IST_WRITE_FIXTURE set; fixture must be resettable outside the UI</t>
+          <t>Uses @axe-core/playwright 4.13.0</t>
         </is>
       </c>
       <c r="K67" s="2" t="inlineStr">
         <is>
-          <t>1. Search +5 years
-2. Compare unselected rows with pre-save snapshot</t>
+          <t>1. Search fixture
+2. Run axe WCAG 2.1 AA, excluding the 3 search dropdowns</t>
         </is>
       </c>
       <c r="L67" s="2" t="inlineStr">
         <is>
-          <t>Unselected rows identical</t>
+          <t>No serious/critical violations</t>
         </is>
       </c>
       <c r="M67" s="2" t="inlineStr">
         <is>
-          <t>NM-4025 trace: TC-IT-33</t>
+          <t>Dropdown labels accepted as-is</t>
         </is>
       </c>
     </row>
@@ -5209,7 +5201,7 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Audit CreateUser and ModUser record the signed-in user</t>
+          <t>Page stays usable at laptop 1366×768</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -5225,19 +5217,19 @@
       <c r="E68" s="2" t="inlineStr">
         <is>
           <t>User: automation user (Tax FULL_ACCESS)
-Office: Office 1101
-Search: IST_WRITE_FIXTURE (disposable)
+Office: Office 1101 (Corporate)
+Search: Mexico / VAT / Baja California
 Application: Navigator</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Responsive</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
@@ -5252,24 +5244,21 @@
       </c>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t>REAL WRITE (insert-only). Runs only with IST_ALLOW_WRITES=true and IST_WRITE_FIXTURE set; fixture must be resettable outside the UI</t>
+          <t>Page opened fresh; no network mocks; non-mutating</t>
         </is>
       </c>
       <c r="K68" s="2" t="inlineStr">
         <is>
-          <t>1. Search at new date, capture response</t>
+          <t>1. Viewport 1366×768
+2. Search fixture</t>
         </is>
       </c>
       <c r="L68" s="2" t="inlineStr">
         <is>
-          <t>CreateUser/ModUser = signed-in user (skips if not exposed)</t>
-        </is>
-      </c>
-      <c r="M68" s="2" t="inlineStr">
-        <is>
-          <t>NM-4025 trace: TC-IT-36</t>
-        </is>
-      </c>
+          <t>Search, Apply, Save reachable; no page sideways scroll</t>
+        </is>
+      </c>
+      <c r="M68" s="2" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -5279,7 +5268,7 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>A read-only tax user can view configurations but cannot Apply or Save</t>
+          <t>Page stays usable at tablet 1024×768</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
@@ -5294,19 +5283,20 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>User: IST_READONLY account (Tax READ only)
-Office: Office 1101
+          <t>User: automation user (Tax FULL_ACCESS)
+Office: Office 1101 (Corporate)
+Search: Mexico / VAT / Baja California
 Application: Navigator</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Responsive</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
@@ -5321,26 +5311,21 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>Needs IST_READONLY_USERNAME/PASSWORD</t>
+          <t>Page opened fresh; no network mocks; non-mutating</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr">
         <is>
-          <t>1. Sign in read-only
-2. Search fixture
-3. Try to select a row</t>
+          <t>1. Viewport 1024×768
+2. Search fixture</t>
         </is>
       </c>
       <c r="L69" s="2" t="inlineStr">
         <is>
-          <t>Rows visible; Apply and Save never enabled</t>
-        </is>
-      </c>
-      <c r="M69" s="2" t="inlineStr">
-        <is>
-          <t>NM-4025 trace: TC-IT-07</t>
-        </is>
-      </c>
+          <t>Search, Apply, Save reachable; no page sideways scroll</t>
+        </is>
+      </c>
+      <c r="M69" s="2" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -5350,7 +5335,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>A user without tax permission sees no menu entry and is refused on the direct route</t>
+          <t>Reset restores the approved defaults</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -5365,19 +5350,20 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>User: IST_NOACCESS account (no Tax permission)
-Office: Office 1101
+          <t>User: automation user (Tax FULL_ACCESS)
+Office: Office 1101 (Corporate)
+Search: Mexico / VAT / Baja California
 Application: Navigator</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Functional</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
@@ -5392,1226 +5378,385 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>Needs IST_NOACCESS_USERNAME/PASSWORD</t>
+          <t>Expected result is an assumption pending NM-4025 §14.2 confirmation (@needs-confirmation)</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr">
-        <is>
-          <t>1. Sign in without Tax permission
-2. Open Tax menu
-3. Open route directly</t>
-        </is>
-      </c>
-      <c r="L70" s="2" t="inlineStr">
-        <is>
-          <t>No menu entry; screen never renders</t>
-        </is>
-      </c>
-      <c r="M70" s="2" t="inlineStr">
-        <is>
-          <t>NM-4025 trace: TC-IT-09</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="2" t="inlineStr">
-        <is>
-          <t>TC-TAX-IST-070</t>
-        </is>
-      </c>
-      <c r="B71" s="2" t="inlineStr">
-        <is>
-          <t>Without a session the page sends the user to sign in</t>
-        </is>
-      </c>
-      <c r="C71" s="2" t="inlineStr">
-        <is>
-          <t>taxes</t>
-        </is>
-      </c>
-      <c r="D71" s="2" t="inlineStr">
-        <is>
-          <t>international_tax_setup</t>
-        </is>
-      </c>
-      <c r="E71" s="2" t="inlineStr">
-        <is>
-          <t>User: none (empty browser context)
-Application: Navigator</t>
-        </is>
-      </c>
-      <c r="F71" s="2" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="G71" s="2" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="H71" s="2" t="inlineStr">
-        <is>
-          <t>Automated</t>
-        </is>
-      </c>
-      <c r="I71" s="2" t="inlineStr">
-        <is>
-          <t>Automated</t>
-        </is>
-      </c>
-      <c r="J71" s="2" t="inlineStr">
-        <is>
-          <t>Page opened fresh; no network mocks; non-mutating</t>
-        </is>
-      </c>
-      <c r="K71" s="2" t="inlineStr">
-        <is>
-          <t>1. Open route with no session</t>
-        </is>
-      </c>
-      <c r="L71" s="2" t="inlineStr">
-        <is>
-          <t>Redirect to /auth/sign-in with callbackUrl; no grid</t>
-        </is>
-      </c>
-      <c r="M71" s="2" t="inlineStr">
-        <is>
-          <t>NM-4025 trace: TC-IT-09</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="2" t="inlineStr">
-        <is>
-          <t>TC-TAX-IST-071</t>
-        </is>
-      </c>
-      <c r="B72" s="2" t="inlineStr">
-        <is>
-          <t>A save sent without a session is refused and writes nothing</t>
-        </is>
-      </c>
-      <c r="C72" s="2" t="inlineStr">
-        <is>
-          <t>taxes</t>
-        </is>
-      </c>
-      <c r="D72" s="2" t="inlineStr">
-        <is>
-          <t>international_tax_setup</t>
-        </is>
-      </c>
-      <c r="E72" s="2" t="inlineStr">
-        <is>
-          <t>User: automation user (Tax FULL_ACCESS)
-Office: Office 1101
-Search: IST_WRITE_FIXTURE (disposable)
-Application: Navigator</t>
-        </is>
-      </c>
-      <c r="F72" s="2" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="G72" s="2" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="H72" s="2" t="inlineStr">
-        <is>
-          <t>Automated</t>
-        </is>
-      </c>
-      <c r="I72" s="2" t="inlineStr">
-        <is>
-          <t>Automated</t>
-        </is>
-      </c>
-      <c r="J72" s="2" t="inlineStr">
-        <is>
-          <t>REAL WRITE (insert-only). Runs only with IST_ALLOW_WRITES=true and IST_WRITE_FIXTURE set; fixture must be resettable outside the UI; payload dated = latest stored (double-safe)</t>
-        </is>
-      </c>
-      <c r="K72" s="2" t="inlineStr">
-        <is>
-          <t>1. Capture a save (held)
-2. Replay it with no session
-3. Search +5 years</t>
-        </is>
-      </c>
-      <c r="L72" s="2" t="inlineStr">
-        <is>
-          <t>Not a plain 200; fixture unchanged</t>
-        </is>
-      </c>
-      <c r="M72" s="2" t="inlineStr">
-        <is>
-          <t>NM-4025 §5.3</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="2" t="inlineStr">
-        <is>
-          <t>TC-TAX-IST-072</t>
-        </is>
-      </c>
-      <c r="B73" s="2" t="inlineStr">
-        <is>
-          <t>A save sent by a read-only user is refused and writes nothing</t>
-        </is>
-      </c>
-      <c r="C73" s="2" t="inlineStr">
-        <is>
-          <t>taxes</t>
-        </is>
-      </c>
-      <c r="D73" s="2" t="inlineStr">
-        <is>
-          <t>international_tax_setup</t>
-        </is>
-      </c>
-      <c r="E73" s="2" t="inlineStr">
-        <is>
-          <t>User: automation user (Tax FULL_ACCESS)
-Office: Office 1101
-Search: IST_WRITE_FIXTURE (disposable)
-Application: Navigator</t>
-        </is>
-      </c>
-      <c r="F73" s="2" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="G73" s="2" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="H73" s="2" t="inlineStr">
-        <is>
-          <t>Automated</t>
-        </is>
-      </c>
-      <c r="I73" s="2" t="inlineStr">
-        <is>
-          <t>Automated</t>
-        </is>
-      </c>
-      <c r="J73" s="2" t="inlineStr">
-        <is>
-          <t>REAL WRITE (insert-only). Runs only with IST_ALLOW_WRITES=true and IST_WRITE_FIXTURE set; fixture must be resettable outside the UI; needs read-only account</t>
-        </is>
-      </c>
-      <c r="K73" s="2" t="inlineStr">
-        <is>
-          <t>1. Capture a save (held)
-2. Replay with read-only session
-3. Search +5 years</t>
-        </is>
-      </c>
-      <c r="L73" s="2" t="inlineStr">
-        <is>
-          <t>Not a plain 200; fixture unchanged</t>
-        </is>
-      </c>
-      <c r="M73" s="2" t="inlineStr">
-        <is>
-          <t>NM-4025 §5.3</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="2" t="inlineStr">
-        <is>
-          <t>TC-TAX-IST-073</t>
-        </is>
-      </c>
-      <c r="B74" s="2" t="inlineStr">
-        <is>
-          <t>A save attempted after the session expires writes nothing</t>
-        </is>
-      </c>
-      <c r="C74" s="2" t="inlineStr">
-        <is>
-          <t>taxes</t>
-        </is>
-      </c>
-      <c r="D74" s="2" t="inlineStr">
-        <is>
-          <t>international_tax_setup</t>
-        </is>
-      </c>
-      <c r="E74" s="2" t="inlineStr">
-        <is>
-          <t>User: automation user (Tax FULL_ACCESS)
-Office: Office 1101
-Search: IST_WRITE_FIXTURE (disposable)
-Application: Navigator</t>
-        </is>
-      </c>
-      <c r="F74" s="2" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="G74" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H74" s="2" t="inlineStr">
-        <is>
-          <t>Automated</t>
-        </is>
-      </c>
-      <c r="I74" s="2" t="inlineStr">
-        <is>
-          <t>Automated</t>
-        </is>
-      </c>
-      <c r="J74" s="2" t="inlineStr">
-        <is>
-          <t>REAL WRITE (insert-only). Runs only with IST_ALLOW_WRITES=true and IST_WRITE_FIXTURE set; fixture must be resettable outside the UI; payload dated = latest stored (double-safe)</t>
-        </is>
-      </c>
-      <c r="K74" s="2" t="inlineStr">
-        <is>
-          <t>1. Stage in a second context
-2. Clear its cookies
-3. Save
-4. Search +5 years</t>
-        </is>
-      </c>
-      <c r="L74" s="2" t="inlineStr">
-        <is>
-          <t>Fixture unchanged</t>
-        </is>
-      </c>
-      <c r="M74" s="2" t="inlineStr">
-        <is>
-          <t>Session expiry mid-edit</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="2" t="inlineStr">
-        <is>
-          <t>TC-TAX-IST-074</t>
-        </is>
-      </c>
-      <c r="B75" s="2" t="inlineStr">
-        <is>
-          <t>Every search and update control has an accessible name</t>
-        </is>
-      </c>
-      <c r="C75" s="2" t="inlineStr">
-        <is>
-          <t>taxes</t>
-        </is>
-      </c>
-      <c r="D75" s="2" t="inlineStr">
-        <is>
-          <t>international_tax_setup</t>
-        </is>
-      </c>
-      <c r="E75" s="2" t="inlineStr">
-        <is>
-          <t>User: automation user (Tax FULL_ACCESS)
-Office: Office 1101 (Corporate)
-Search: Mexico / VAT / Baja California
-Application: Navigator</t>
-        </is>
-      </c>
-      <c r="F75" s="2" t="inlineStr">
-        <is>
-          <t>Accessibility</t>
-        </is>
-      </c>
-      <c r="G75" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H75" s="2" t="inlineStr">
-        <is>
-          <t>Automated</t>
-        </is>
-      </c>
-      <c r="I75" s="2" t="inlineStr">
-        <is>
-          <t>Automated</t>
-        </is>
-      </c>
-      <c r="J75" s="2" t="inlineStr">
-        <is>
-          <t>KNOWN DEFECT — test.fail(BUG-TAX-IST-003)</t>
-        </is>
-      </c>
-      <c r="K75" s="2" t="inlineStr">
-        <is>
-          <t>1. Read accessible names of every control</t>
-        </is>
-      </c>
-      <c r="L75" s="2" t="inlineStr">
-        <is>
-          <t>None empty; names match their labels</t>
-        </is>
-      </c>
-      <c r="M75" s="2" t="inlineStr">
-        <is>
-          <t>WCAG 4.1.2 (BUG-TAX-IST-003)</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="2" t="inlineStr">
-        <is>
-          <t>TC-TAX-IST-075</t>
-        </is>
-      </c>
-      <c r="B76" s="2" t="inlineStr">
-        <is>
-          <t>Row checkboxes can be operated with the keyboard</t>
-        </is>
-      </c>
-      <c r="C76" s="2" t="inlineStr">
-        <is>
-          <t>taxes</t>
-        </is>
-      </c>
-      <c r="D76" s="2" t="inlineStr">
-        <is>
-          <t>international_tax_setup</t>
-        </is>
-      </c>
-      <c r="E76" s="2" t="inlineStr">
-        <is>
-          <t>User: automation user (Tax FULL_ACCESS)
-Office: Office 1101 (Corporate)
-Search: Mexico / VAT / Baja California
-Application: Navigator</t>
-        </is>
-      </c>
-      <c r="F76" s="2" t="inlineStr">
-        <is>
-          <t>Accessibility</t>
-        </is>
-      </c>
-      <c r="G76" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H76" s="2" t="inlineStr">
-        <is>
-          <t>Automated</t>
-        </is>
-      </c>
-      <c r="I76" s="2" t="inlineStr">
-        <is>
-          <t>Automated</t>
-        </is>
-      </c>
-      <c r="J76" s="2" t="inlineStr">
-        <is>
-          <t>Page opened fresh; no network mocks; non-mutating</t>
-        </is>
-      </c>
-      <c r="K76" s="2" t="inlineStr">
-        <is>
-          <t>1. Focus a row checkbox
-2. Press Space twice</t>
-        </is>
-      </c>
-      <c r="L76" s="2" t="inlineStr">
-        <is>
-          <t>Selected then cleared</t>
-        </is>
-      </c>
-      <c r="M76" s="2" t="inlineStr">
-        <is>
-          <t>WCAG 2.1.1</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="2" t="inlineStr">
-        <is>
-          <t>TC-TAX-IST-076</t>
-        </is>
-      </c>
-      <c r="B77" s="2" t="inlineStr">
-        <is>
-          <t>Tab order through the search panel follows the visual order</t>
-        </is>
-      </c>
-      <c r="C77" s="2" t="inlineStr">
-        <is>
-          <t>taxes</t>
-        </is>
-      </c>
-      <c r="D77" s="2" t="inlineStr">
-        <is>
-          <t>international_tax_setup</t>
-        </is>
-      </c>
-      <c r="E77" s="2" t="inlineStr">
-        <is>
-          <t>User: automation user (Tax FULL_ACCESS)
-Office: Office 1101 (Corporate)
-Search: Mexico / VAT / Baja California
-Application: Navigator</t>
-        </is>
-      </c>
-      <c r="F77" s="2" t="inlineStr">
-        <is>
-          <t>Accessibility</t>
-        </is>
-      </c>
-      <c r="G77" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H77" s="2" t="inlineStr">
-        <is>
-          <t>Automated</t>
-        </is>
-      </c>
-      <c r="I77" s="2" t="inlineStr">
-        <is>
-          <t>Automated</t>
-        </is>
-      </c>
-      <c r="J77" s="2" t="inlineStr">
-        <is>
-          <t>Page opened fresh; no network mocks; non-mutating</t>
-        </is>
-      </c>
-      <c r="K77" s="2" t="inlineStr">
-        <is>
-          <t>1. Focus Country
-2. Tab through the panel</t>
-        </is>
-      </c>
-      <c r="L77" s="2" t="inlineStr">
-        <is>
-          <t>Tax Group → Province → Effective Date → Reset → Search</t>
-        </is>
-      </c>
-      <c r="M77" s="2" t="inlineStr">
-        <is>
-          <t>WCAG 2.4.3</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="2" t="inlineStr">
-        <is>
-          <t>TC-TAX-IST-077</t>
-        </is>
-      </c>
-      <c r="B78" s="2" t="inlineStr">
-        <is>
-          <t>No untranslated i18n key is visible on the page</t>
-        </is>
-      </c>
-      <c r="C78" s="2" t="inlineStr">
-        <is>
-          <t>taxes</t>
-        </is>
-      </c>
-      <c r="D78" s="2" t="inlineStr">
-        <is>
-          <t>international_tax_setup</t>
-        </is>
-      </c>
-      <c r="E78" s="2" t="inlineStr">
-        <is>
-          <t>User: automation user (Tax FULL_ACCESS)
-Office: Office 1101 (Corporate)
-Search: Mexico / VAT / Baja California
-Application: Navigator</t>
-        </is>
-      </c>
-      <c r="F78" s="2" t="inlineStr">
-        <is>
-          <t>Localisation</t>
-        </is>
-      </c>
-      <c r="G78" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H78" s="2" t="inlineStr">
-        <is>
-          <t>Automated</t>
-        </is>
-      </c>
-      <c r="I78" s="2" t="inlineStr">
-        <is>
-          <t>Automated</t>
-        </is>
-      </c>
-      <c r="J78" s="2" t="inlineStr">
-        <is>
-          <t>Page opened fresh; no network mocks; non-mutating</t>
-        </is>
-      </c>
-      <c r="K78" s="2" t="inlineStr">
-        <is>
-          <t>1. Search fixture
-2. Scan page text</t>
-        </is>
-      </c>
-      <c r="L78" s="2" t="inlineStr">
-        <is>
-          <t>No dotted i18n keys</t>
-        </is>
-      </c>
-      <c r="M78" s="2" t="inlineStr"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="2" t="inlineStr">
-        <is>
-          <t>TC-TAX-IST-078</t>
-        </is>
-      </c>
-      <c r="B79" s="2" t="inlineStr">
-        <is>
-          <t>Automated WCAG 2.1 AA scan finds no serious or critical violations</t>
-        </is>
-      </c>
-      <c r="C79" s="2" t="inlineStr">
-        <is>
-          <t>taxes</t>
-        </is>
-      </c>
-      <c r="D79" s="2" t="inlineStr">
-        <is>
-          <t>international_tax_setup</t>
-        </is>
-      </c>
-      <c r="E79" s="2" t="inlineStr">
-        <is>
-          <t>User: automation user (Tax FULL_ACCESS)
-Office: Office 1101 (Corporate)
-Search: Mexico / VAT / Baja California
-Application: Navigator</t>
-        </is>
-      </c>
-      <c r="F79" s="2" t="inlineStr">
-        <is>
-          <t>Accessibility</t>
-        </is>
-      </c>
-      <c r="G79" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H79" s="2" t="inlineStr">
-        <is>
-          <t>Automated</t>
-        </is>
-      </c>
-      <c r="I79" s="2" t="inlineStr">
-        <is>
-          <t>Automated</t>
-        </is>
-      </c>
-      <c r="J79" s="2" t="inlineStr">
-        <is>
-          <t>Uses @axe-core/playwright 4.13.0; KNOWN DEFECT — test.fail(BUG-TAX-IST-003)</t>
-        </is>
-      </c>
-      <c r="K79" s="2" t="inlineStr">
-        <is>
-          <t>1. Search fixture
-2. Run axe WCAG 2.1 AA</t>
-        </is>
-      </c>
-      <c r="L79" s="2" t="inlineStr">
-        <is>
-          <t>No serious/critical violations</t>
-        </is>
-      </c>
-      <c r="M79" s="2" t="inlineStr">
-        <is>
-          <t>axe button-name critical on the 3 dropdowns (BUG-TAX-IST-003)</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="2" t="inlineStr">
-        <is>
-          <t>TC-TAX-IST-079</t>
-        </is>
-      </c>
-      <c r="B80" s="2" t="inlineStr">
-        <is>
-          <t>Page stays usable at laptop 1366×768</t>
-        </is>
-      </c>
-      <c r="C80" s="2" t="inlineStr">
-        <is>
-          <t>taxes</t>
-        </is>
-      </c>
-      <c r="D80" s="2" t="inlineStr">
-        <is>
-          <t>international_tax_setup</t>
-        </is>
-      </c>
-      <c r="E80" s="2" t="inlineStr">
-        <is>
-          <t>User: automation user (Tax FULL_ACCESS)
-Office: Office 1101 (Corporate)
-Search: Mexico / VAT / Baja California
-Application: Navigator</t>
-        </is>
-      </c>
-      <c r="F80" s="2" t="inlineStr">
-        <is>
-          <t>Responsive</t>
-        </is>
-      </c>
-      <c r="G80" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H80" s="2" t="inlineStr">
-        <is>
-          <t>Automated</t>
-        </is>
-      </c>
-      <c r="I80" s="2" t="inlineStr">
-        <is>
-          <t>Automated</t>
-        </is>
-      </c>
-      <c r="J80" s="2" t="inlineStr">
-        <is>
-          <t>Page opened fresh; no network mocks; non-mutating</t>
-        </is>
-      </c>
-      <c r="K80" s="2" t="inlineStr">
-        <is>
-          <t>1. Viewport 1366×768
-2. Search fixture</t>
-        </is>
-      </c>
-      <c r="L80" s="2" t="inlineStr">
-        <is>
-          <t>Search, Apply, Save reachable; no page sideways scroll</t>
-        </is>
-      </c>
-      <c r="M80" s="2" t="inlineStr"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="2" t="inlineStr">
-        <is>
-          <t>TC-TAX-IST-080</t>
-        </is>
-      </c>
-      <c r="B81" s="2" t="inlineStr">
-        <is>
-          <t>Page stays usable at tablet 1024×768</t>
-        </is>
-      </c>
-      <c r="C81" s="2" t="inlineStr">
-        <is>
-          <t>taxes</t>
-        </is>
-      </c>
-      <c r="D81" s="2" t="inlineStr">
-        <is>
-          <t>international_tax_setup</t>
-        </is>
-      </c>
-      <c r="E81" s="2" t="inlineStr">
-        <is>
-          <t>User: automation user (Tax FULL_ACCESS)
-Office: Office 1101 (Corporate)
-Search: Mexico / VAT / Baja California
-Application: Navigator</t>
-        </is>
-      </c>
-      <c r="F81" s="2" t="inlineStr">
-        <is>
-          <t>Responsive</t>
-        </is>
-      </c>
-      <c r="G81" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H81" s="2" t="inlineStr">
-        <is>
-          <t>Automated</t>
-        </is>
-      </c>
-      <c r="I81" s="2" t="inlineStr">
-        <is>
-          <t>Automated</t>
-        </is>
-      </c>
-      <c r="J81" s="2" t="inlineStr">
-        <is>
-          <t>Page opened fresh; no network mocks; non-mutating</t>
-        </is>
-      </c>
-      <c r="K81" s="2" t="inlineStr">
-        <is>
-          <t>1. Viewport 1024×768
-2. Search fixture</t>
-        </is>
-      </c>
-      <c r="L81" s="2" t="inlineStr">
-        <is>
-          <t>Search, Apply, Save reachable; no page sideways scroll</t>
-        </is>
-      </c>
-      <c r="M81" s="2" t="inlineStr"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="2" t="inlineStr">
-        <is>
-          <t>TC-TAX-IST-081</t>
-        </is>
-      </c>
-      <c r="B82" s="2" t="inlineStr">
-        <is>
-          <t>Reset restores the approved defaults</t>
-        </is>
-      </c>
-      <c r="C82" s="2" t="inlineStr">
-        <is>
-          <t>taxes</t>
-        </is>
-      </c>
-      <c r="D82" s="2" t="inlineStr">
-        <is>
-          <t>international_tax_setup</t>
-        </is>
-      </c>
-      <c r="E82" s="2" t="inlineStr">
-        <is>
-          <t>User: automation user (Tax FULL_ACCESS)
-Office: Office 1101 (Corporate)
-Search: Mexico / VAT / Baja California
-Application: Navigator</t>
-        </is>
-      </c>
-      <c r="F82" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="G82" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H82" s="2" t="inlineStr">
-        <is>
-          <t>Automated</t>
-        </is>
-      </c>
-      <c r="I82" s="2" t="inlineStr">
-        <is>
-          <t>Automated</t>
-        </is>
-      </c>
-      <c r="J82" s="2" t="inlineStr">
-        <is>
-          <t>Expected result is an assumption pending NM-4025 §14.2 confirmation (@needs-confirmation)</t>
-        </is>
-      </c>
-      <c r="K82" s="2" t="inlineStr">
         <is>
           <t>1. Search fixture at an old date
 2. Click Reset
 3. Stage a change, click Reset</t>
         </is>
       </c>
-      <c r="L82" s="2" t="inlineStr">
+      <c r="L70" s="2" t="inlineStr">
         <is>
           <t>Province cleared, date today, grid empty, no auto-search, Country/Tax Group kept; dirty Reset warns</t>
         </is>
       </c>
-      <c r="M82" s="2" t="inlineStr">
+      <c r="M70" s="2" t="inlineStr">
         <is>
           <t>NM-4025 trace: TC-IT-39; §6.4 (characterised live)</t>
         </is>
       </c>
     </row>
-    <row r="83">
-      <c r="A83" s="2" t="inlineStr">
-        <is>
-          <t>TC-TAX-IST-082</t>
-        </is>
-      </c>
-      <c r="B83" s="2" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>TC-TAX-IST-070</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
         <is>
           <t>Header select-all selects the approved scope</t>
         </is>
       </c>
-      <c r="C83" s="2" t="inlineStr">
-        <is>
-          <t>taxes</t>
-        </is>
-      </c>
-      <c r="D83" s="2" t="inlineStr">
-        <is>
-          <t>international_tax_setup</t>
-        </is>
-      </c>
-      <c r="E83" s="2" t="inlineStr">
-        <is>
-          <t>User: automation user (Tax FULL_ACCESS)
-Office: Office 1101 (Corporate)
-Search: Mexico / VAT / Baja California
-Application: Navigator</t>
-        </is>
-      </c>
-      <c r="F83" s="2" t="inlineStr">
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>taxes</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>international_tax_setup</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>User: automation user (Tax FULL_ACCESS)
+Office: Office 1101 (Corporate)
+Search: Mexico / VAT / Baja California
+Application: Navigator</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="G83" s="2" t="inlineStr">
+      <c r="G71" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H83" s="2" t="inlineStr">
-        <is>
-          <t>Automated</t>
-        </is>
-      </c>
-      <c r="I83" s="2" t="inlineStr">
-        <is>
-          <t>Automated</t>
-        </is>
-      </c>
-      <c r="J83" s="2" t="inlineStr">
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="J71" s="2" t="inlineStr">
         <is>
           <t>Expected result is an assumption pending NM-4025 §14.2 confirmation (@needs-confirmation)</t>
         </is>
       </c>
-      <c r="K83" s="2" t="inlineStr">
+      <c r="K71" s="2" t="inlineStr">
         <is>
           <t>1. Tick header select-all
 2. Clear one row
 3. Tick header again</t>
         </is>
       </c>
-      <c r="L83" s="2" t="inlineStr">
+      <c r="L71" s="2" t="inlineStr">
         <is>
           <t>All rows selected; header unticks on partial selection; all again</t>
         </is>
       </c>
-      <c r="M83" s="2" t="inlineStr">
+      <c r="M71" s="2" t="inlineStr">
         <is>
           <t>NM-4025 §4.1 (characterised live; no indeterminate state)</t>
         </is>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" s="2" t="inlineStr">
-        <is>
-          <t>TC-TAX-IST-083</t>
-        </is>
-      </c>
-      <c r="B84" s="2" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>TC-TAX-IST-071</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
         <is>
           <t>Apply with no selection shows the approved feedback</t>
         </is>
       </c>
-      <c r="C84" s="2" t="inlineStr">
-        <is>
-          <t>taxes</t>
-        </is>
-      </c>
-      <c r="D84" s="2" t="inlineStr">
-        <is>
-          <t>international_tax_setup</t>
-        </is>
-      </c>
-      <c r="E84" s="2" t="inlineStr">
-        <is>
-          <t>User: automation user (Tax FULL_ACCESS)
-Office: Office 1101 (Corporate)
-Search: Mexico / VAT / Baja California
-Application: Navigator</t>
-        </is>
-      </c>
-      <c r="F84" s="2" t="inlineStr">
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>taxes</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>international_tax_setup</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>User: automation user (Tax FULL_ACCESS)
+Office: Office 1101 (Corporate)
+Search: Mexico / VAT / Baja California
+Application: Navigator</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="G84" s="2" t="inlineStr">
+      <c r="G72" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H84" s="2" t="inlineStr">
-        <is>
-          <t>Automated</t>
-        </is>
-      </c>
-      <c r="I84" s="2" t="inlineStr">
-        <is>
-          <t>Automated</t>
-        </is>
-      </c>
-      <c r="J84" s="2" t="inlineStr">
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="J72" s="2" t="inlineStr">
         <is>
           <t>Expected result is an assumption pending NM-4025 §14.2 confirmation (@needs-confirmation)</t>
         </is>
       </c>
-      <c r="K84" s="2" t="inlineStr">
+      <c r="K72" s="2" t="inlineStr">
         <is>
           <t>1. Enter a Rate with nothing selected
 2. Select a row</t>
         </is>
       </c>
-      <c r="L84" s="2" t="inlineStr">
+      <c r="L72" s="2" t="inlineStr">
         <is>
           <t>Apply disabled without selection, enabled with one</t>
         </is>
       </c>
-      <c r="M84" s="2" t="inlineStr">
+      <c r="M72" s="2" t="inlineStr">
         <is>
           <t>NM-4025 trace: TC-IT-24 (characterised live)</t>
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" s="2" t="inlineStr">
-        <is>
-          <t>TC-TAX-IST-084</t>
-        </is>
-      </c>
-      <c r="B85" s="2" t="inlineStr">
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>TC-TAX-IST-072</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
         <is>
           <t>Rate minimum, maximum, precision and rounding rules are enforced</t>
         </is>
       </c>
-      <c r="C85" s="2" t="inlineStr">
-        <is>
-          <t>taxes</t>
-        </is>
-      </c>
-      <c r="D85" s="2" t="inlineStr">
-        <is>
-          <t>international_tax_setup</t>
-        </is>
-      </c>
-      <c r="E85" s="2" t="inlineStr">
-        <is>
-          <t>User: automation user (Tax FULL_ACCESS)
-Office: Office 1101 (Corporate)
-Search: Mexico / VAT / Baja California
-Application: Navigator</t>
-        </is>
-      </c>
-      <c r="F85" s="2" t="inlineStr">
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>taxes</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>international_tax_setup</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>User: automation user (Tax FULL_ACCESS)
+Office: Office 1101 (Corporate)
+Search: Mexico / VAT / Baja California
+Application: Navigator</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
         <is>
           <t>Boundary</t>
         </is>
       </c>
-      <c r="G85" s="2" t="inlineStr">
+      <c r="G73" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H85" s="2" t="inlineStr">
-        <is>
-          <t>Automated</t>
-        </is>
-      </c>
-      <c r="I85" s="2" t="inlineStr">
-        <is>
-          <t>Automated</t>
-        </is>
-      </c>
-      <c r="J85" s="2" t="inlineStr">
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="I73" s="2" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="J73" s="2" t="inlineStr">
         <is>
           <t>Expected result is an assumption pending NM-4025 §14.2 confirmation (@needs-confirmation)</t>
         </is>
       </c>
-      <c r="K85" s="2" t="inlineStr">
+      <c r="K73" s="2" t="inlineStr">
         <is>
           <t>1. Type abc, -5, 150, 99999999, 1.23456, 0.0001 into Rate</t>
         </is>
       </c>
-      <c r="L85" s="2" t="inlineStr">
+      <c r="L73" s="2" t="inlineStr">
         <is>
           <t>Only non-negative numbers kept; oversized values capped at 100</t>
         </is>
       </c>
-      <c r="M85" s="2" t="inlineStr">
+      <c r="M73" s="2" t="inlineStr">
         <is>
           <t>NM-4025 §14.1 / Q4 (characterised live; precision recorded only)</t>
         </is>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" s="2" t="inlineStr">
-        <is>
-          <t>TC-TAX-IST-085</t>
-        </is>
-      </c>
-      <c r="B86" s="2" t="inlineStr">
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>TC-TAX-IST-073</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
         <is>
           <t>Blank update fields follow the approved partial-update contract</t>
         </is>
       </c>
-      <c r="C86" s="2" t="inlineStr">
-        <is>
-          <t>taxes</t>
-        </is>
-      </c>
-      <c r="D86" s="2" t="inlineStr">
-        <is>
-          <t>international_tax_setup</t>
-        </is>
-      </c>
-      <c r="E86" s="2" t="inlineStr">
-        <is>
-          <t>User: automation user (Tax FULL_ACCESS)
-Office: Office 1101 (Corporate)
-Search: Mexico / VAT / Baja California
-Application: Navigator</t>
-        </is>
-      </c>
-      <c r="F86" s="2" t="inlineStr">
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>taxes</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>international_tax_setup</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>User: automation user (Tax FULL_ACCESS)
+Office: Office 1101 (Corporate)
+Search: Mexico / VAT / Baja California
+Application: Navigator</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="G86" s="2" t="inlineStr">
+      <c r="G74" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H86" s="2" t="inlineStr">
-        <is>
-          <t>Automated</t>
-        </is>
-      </c>
-      <c r="I86" s="2" t="inlineStr">
-        <is>
-          <t>Automated</t>
-        </is>
-      </c>
-      <c r="J86" s="2" t="inlineStr">
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="J74" s="2" t="inlineStr">
         <is>
           <t>Expected result is an assumption pending NM-4025 §14.2 confirmation (@needs-confirmation)</t>
         </is>
       </c>
-      <c r="K86" s="2" t="inlineStr">
+      <c r="K74" s="2" t="inlineStr">
         <is>
           <t>1. Untick Is Commission Taxable?
 2. Apply to a row that has it</t>
         </is>
       </c>
-      <c r="L86" s="2" t="inlineStr">
+      <c r="L74" s="2" t="inlineStr">
         <is>
           <t>Row commission flag cleared — Apply writes every field</t>
         </is>
       </c>
-      <c r="M86" s="2" t="inlineStr">
+      <c r="M74" s="2" t="inlineStr">
         <is>
           <t>NM-4025 Q5 (characterised live)</t>
         </is>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" s="2" t="inlineStr">
-        <is>
-          <t>TC-TAX-IST-086</t>
-        </is>
-      </c>
-      <c r="B87" s="2" t="inlineStr">
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>TC-TAX-IST-074</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
         <is>
           <t>Edit rights follow the approved office scope</t>
         </is>
       </c>
-      <c r="C87" s="2" t="inlineStr">
-        <is>
-          <t>taxes</t>
-        </is>
-      </c>
-      <c r="D87" s="2" t="inlineStr">
-        <is>
-          <t>international_tax_setup</t>
-        </is>
-      </c>
-      <c r="E87" s="2" t="inlineStr">
-        <is>
-          <t>User: automation user (Tax FULL_ACCESS)
-Office: Office 1101 (Corporate)
-Search: Mexico / VAT / Baja California
-Application: Navigator</t>
-        </is>
-      </c>
-      <c r="F87" s="2" t="inlineStr">
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>taxes</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>international_tax_setup</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>User: automation user (Tax FULL_ACCESS)
+Office: Office 1101 (Corporate)
+Search: Mexico / VAT / Baja California
+Application: Navigator</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
         <is>
           <t>Security</t>
         </is>
       </c>
-      <c r="G87" s="2" t="inlineStr">
+      <c r="G75" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H87" s="2" t="inlineStr">
-        <is>
-          <t>Automated</t>
-        </is>
-      </c>
-      <c r="I87" s="2" t="inlineStr">
-        <is>
-          <t>Automated</t>
-        </is>
-      </c>
-      <c r="J87" s="2" t="inlineStr">
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="I75" s="2" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="J75" s="2" t="inlineStr">
         <is>
           <t>Expected result is an assumption pending NM-4025 §14.2 confirmation (@needs-confirmation)</t>
         </is>
       </c>
-      <c r="K87" s="2" t="inlineStr">
+      <c r="K75" s="2" t="inlineStr">
         <is>
           <t>1. Open from office 2359
 2. Search fixture
 3. Select a row</t>
         </is>
       </c>
-      <c r="L87" s="2" t="inlineStr">
+      <c r="L75" s="2" t="inlineStr">
         <is>
           <t>Rows listed; checkboxes usable; Apply enabled</t>
         </is>
       </c>
-      <c r="M87" s="2" t="inlineStr">
+      <c r="M75" s="2" t="inlineStr">
         <is>
           <t>NM-4025 §5.2 (characterised live)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M87"/>
+  <autoFilter ref="A1:M75"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>